<commit_message>
Move DB connection strings to User Secrets; add Email to employee import
Adds Microsoft.Extensions.Configuration.UserSecrets to hrms-api,
hrms-adms-api, and hrms.Infrastructure so local connection strings no longer
need to live in appsettings.json -- HrmsConnection is blanked out there
accordingly. Also updates the TenantStore DB host in MigrationHrms's
appsettings.json.

Unrelated: EmployeeImportService/the employee import template now support an
Email column.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/hrms-api/wwwroot/Templates/employee_template.xlsx
+++ b/hrms-api/wwwroot/Templates/employee_template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HII admin\Documents\VsCode\hrms-api\hrms-api\wwwroot\Templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{547E4621-5D0D-4EB1-9E30-C586606A8854}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AB31E980-C976-443A-97C4-407DFF1F46B2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{CB0C57D7-EEA7-4E4B-801E-9CD0B5FFF564}"/>
   </bookViews>
@@ -167,7 +167,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="46">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="47">
   <si>
     <t>LastName</t>
   </si>
@@ -306,13 +306,16 @@
   </si>
   <si>
     <t>Monthly</t>
+  </si>
+  <si>
+    <t>Email</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -326,12 +329,6 @@
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="9"/>
-      <color indexed="81"/>
-      <name val="Tahoma"/>
-      <charset val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -758,7 +755,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{38D9F31A-E2EC-4988-BBA0-8862FC76D1CC}">
-  <dimension ref="A1:AI6"/>
+  <dimension ref="A1:AJ6"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="14.5703125" customWidth="1"/>
@@ -792,7 +789,7 @@
     <col min="32" max="32" width="15.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:35" ht="39" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:36" ht="39" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="6" t="s">
         <v>2</v>
       </c>
@@ -829,7 +826,7 @@
       <c r="AD1" s="5"/>
       <c r="AE1" s="5"/>
     </row>
-    <row r="2" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -935,8 +932,11 @@
       <c r="AI2" t="s">
         <v>32</v>
       </c>
+      <c r="AJ2" t="s">
+        <v>46</v>
+      </c>
     </row>
-    <row r="3" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>1</v>
       </c>
@@ -998,7 +998,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="4" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:36" x14ac:dyDescent="0.25">
       <c r="L4" t="s">
         <v>39</v>
       </c>
@@ -1021,7 +1021,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:36" x14ac:dyDescent="0.25">
       <c r="L5" t="s">
         <v>40</v>
       </c>
@@ -1050,7 +1050,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:36" x14ac:dyDescent="0.25">
       <c r="L6" t="s">
         <v>45</v>
       </c>

</xml_diff>

<commit_message>
Restore employee_template.xlsx, reverting an unintended overwrite
The previous commit (b8d97ed) picked up a stray already-staged change to
this file that stripped its per-column cell comments (xl/comments1.xml,
xl/threadedComments/, xl/persons/person.xml) and the VML comment-indicator
drawing (xl/drawings/vmlDrawing1.vml) -- the very comments the template's
own "Instructions:" banner text refers to ("I have also added comments in
certain columns with specific instructions"). That change was never
reviewed or intended as part of the employee-import-preview work; this
restores the file exactly as it was before that commit.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/hrms-api/wwwroot/Templates/employee_template.xlsx
+++ b/hrms-api/wwwroot/Templates/employee_template.xlsx
@@ -1,22 +1,25 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30326"/>
-  <workbookPr/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HII admin\Documents\VsCode\hrms-api\hrms-api\wwwroot\Templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B957B507-6E0E-4516-A937-88DE5587A032}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AB31E980-C976-443A-97C4-407DFF1F46B2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{CB0C57D7-EEA7-4E4B-801E-9CD0B5FFF564}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
+      <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
         <xcalcf:feature name="microsoft.com:RD"/>
@@ -32,149 +35,280 @@
 </workbook>
 </file>
 
+<file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
+  <authors>
+    <author>tc={9BFC5F6E-C6A0-42C0-B8AB-F1F3D1249D2B}</author>
+    <author>tc={79FCC02C-F85F-405C-A566-509890A3EBC9}</author>
+    <author>tc={06C68CE5-F9F3-46D3-97DC-8969C057FDE5}</author>
+    <author>tc={96EB2AF4-8857-453C-84CF-C7D0294A47E1}</author>
+    <author>tc={ED936B87-B4EA-49D2-9847-251F065AD106}</author>
+    <author>tc={861CEFFE-75F3-4A22-A7B0-DE08527FCA28}</author>
+    <author>tc={41A77145-9368-44AE-B73E-F2FA9D9BF935}</author>
+    <author>tc={73102409-9A79-496E-AAB6-27215C458146}</author>
+    <author>tc={C3B48641-F285-4034-95EA-970F81F494AD}</author>
+    <author>tc={A1D30F49-4CC7-4810-8930-31A0E5E3D18D}</author>
+    <author>tc={0D448524-4E4F-4A1C-9A6D-66C1E154C2FC}</author>
+    <author>tc={B19BC939-9062-41D8-A080-1F0317F4D29D}</author>
+    <author>tc={F0E96506-AAF2-49B7-AD58-D5B640AC0623}</author>
+  </authors>
+  <commentList>
+    <comment ref="A2" authorId="0" shapeId="0" xr:uid="{9BFC5F6E-C6A0-42C0-B8AB-F1F3D1249D2B}">
+      <text>
+        <t xml:space="preserve">[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    This is the biometric ID that must be set on the device </t>
+      </text>
+    </comment>
+    <comment ref="H2" authorId="1" shapeId="0" xr:uid="{79FCC02C-F85F-405C-A566-509890A3EBC9}">
+      <text>
+        <t xml:space="preserve">[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Enter the day name in the column, or leave it blank if not applicable </t>
+      </text>
+    </comment>
+    <comment ref="I2" authorId="2" shapeId="0" xr:uid="{06C68CE5-F9F3-46D3-97DC-8969C057FDE5}">
+      <text>
+        <t xml:space="preserve">[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Enter the day name in the column, or leave it blank if not applicable </t>
+      </text>
+    </comment>
+    <comment ref="N2" authorId="3" shapeId="0" xr:uid="{96EB2AF4-8857-453C-84CF-C7D0294A47E1}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    End of Month</t>
+      </text>
+    </comment>
+    <comment ref="P2" authorId="4" shapeId="0" xr:uid="{ED936B87-B4EA-49D2-9847-251F065AD106}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    End of Month</t>
+      </text>
+    </comment>
+    <comment ref="R2" authorId="5" shapeId="0" xr:uid="{861CEFFE-75F3-4A22-A7B0-DE08527FCA28}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    End of Month</t>
+      </text>
+    </comment>
+    <comment ref="T2" authorId="6" shapeId="0" xr:uid="{41A77145-9368-44AE-B73E-F2FA9D9BF935}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    End of Month</t>
+      </text>
+    </comment>
+    <comment ref="U2" authorId="7" shapeId="0" xr:uid="{73102409-9A79-496E-AAB6-27215C458146}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    You can Enter any Time Shift name here</t>
+      </text>
+    </comment>
+    <comment ref="W2" authorId="8" shapeId="0" xr:uid="{C3B48641-F285-4034-95EA-970F81F494AD}">
+      <text>
+        <t xml:space="preserve">[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Use the same time format shown here. For example, enter 08:00:00 for 8:00 AM and 17:00:00 for 5:00 PM. If the time crosses into the next day, prefix it with 1. before the time. For instance, 1.01:00:00 represents 1:00 AM on the following day. </t>
+      </text>
+    </comment>
+    <comment ref="Y2" authorId="9" shapeId="0" xr:uid="{A1D30F49-4CC7-4810-8930-31A0E5E3D18D}">
+      <text>
+        <t xml:space="preserve">[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Use the same time format shown here. For example, enter 08:00:00 for 8:00 AM and 17:00:00 for 5:00 PM. If the time crosses into the next day, prefix it with 1. before the time. For instance, 1.01:00:00 represents 1:00 AM on the following day. </t>
+      </text>
+    </comment>
+    <comment ref="Z2" authorId="10" shapeId="0" xr:uid="{0D448524-4E4F-4A1C-9A6D-66C1E154C2FC}">
+      <text>
+        <t xml:space="preserve">[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Use the same time format shown here. For example, enter 08:00:00 for 8:00 AM and 17:00:00 for 5:00 PM. If the time crosses into the next day, prefix it with 1. before the time. For instance, 1.01:00:00 represents 1:00 AM on the following day. 
+</t>
+      </text>
+    </comment>
+    <comment ref="AB2" authorId="11" shapeId="0" xr:uid="{B19BC939-9062-41D8-A080-1F0317F4D29D}">
+      <text>
+        <t xml:space="preserve">[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    This field represents the total working minutes in a day, excluding unpaid breaks. For example, 480 minutes correspond to 8 hours. If an employee is on a compressed schedule, such as 9 hours per day, you must enter the calculation (9 × 60 = 540) to reflect the correct total. </t>
+      </text>
+    </comment>
+    <comment ref="AD2" authorId="12" shapeId="0" xr:uid="{F0E96506-AAF2-49B7-AD58-D5B640AC0623}">
+      <text>
+        <t xml:space="preserve">[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    The Salary Type column defines how an employee’s salary is calculated for the payroll period. It determines whether the computation is based on actual work hours or on a fixed monthly rate.
+Daily and Monthly Variable: Salary is computed based on the employee’s recorded work hours. This means pay is directly tied to attendance and the number of hours worked within the period.
+Monthly Fixed: Salary is calculated based on the employee’s fixed monthly rate. Deductions are applied for lateness, undertime (UT), and absences, but the base salary remains constant regardless of daily work hours.
+By specifying the correct salary type, the system ensures accurate payroll processing and compliance with company policies
+</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="47">
   <si>
+    <t>LastName</t>
+  </si>
+  <si>
+    <t>MiddleName</t>
+  </si>
+  <si>
     <t>Instructions:</t>
+  </si>
+  <si>
+    <t>BioId</t>
+  </si>
+  <si>
+    <t>Branch Code</t>
+  </si>
+  <si>
+    <t>FirstName</t>
+  </si>
+  <si>
+    <t>Suffix</t>
+  </si>
+  <si>
+    <t>Gender</t>
+  </si>
+  <si>
+    <t>Rest Day 1</t>
+  </si>
+  <si>
+    <t>Rest Day 2</t>
+  </si>
+  <si>
+    <t>Department Name</t>
+  </si>
+  <si>
+    <t>Client Name</t>
+  </si>
+  <si>
+    <t>Payroll Group</t>
+  </si>
+  <si>
+    <t>Shift Name</t>
+  </si>
+  <si>
+    <t>Shift Type</t>
+  </si>
+  <si>
+    <t>AMIN</t>
+  </si>
+  <si>
+    <t>AM Out</t>
+  </si>
+  <si>
+    <t>PM In</t>
+  </si>
+  <si>
+    <t>PM OUT</t>
+  </si>
+  <si>
+    <t>Break Duration</t>
+  </si>
+  <si>
+    <t>Max Working Minutes</t>
+  </si>
+  <si>
+    <t>PaidLunchBreak</t>
+  </si>
+  <si>
+    <t>Saturday</t>
+  </si>
+  <si>
+    <t>Sunday</t>
+  </si>
+  <si>
+    <t>Fixed</t>
+  </si>
+  <si>
+    <t>Daysshift - 08:00-17:00</t>
+  </si>
+  <si>
+    <t>8:00:00AM</t>
   </si>
   <si>
     <t>Sample data are provided for each column. Before filling out this template, copy the data starting from the third row down to the last row of your dataset to ensure that all formulas and validations are carried over. I have also added comments in certain columns with
  specific instructions. Finally, remove any extra or blank rows at the end so the system does not read unwanted entries.</t>
   </si>
   <si>
-    <t>BioId</t>
-  </si>
-  <si>
-    <t>Branch Code</t>
-  </si>
-  <si>
-    <t>FirstName</t>
-  </si>
-  <si>
-    <t>MiddleName</t>
-  </si>
-  <si>
-    <t>LastName</t>
-  </si>
-  <si>
-    <t>Suffix</t>
-  </si>
-  <si>
-    <t>Gender</t>
-  </si>
-  <si>
-    <t>Rest Day 1</t>
-  </si>
-  <si>
-    <t>Rest Day 2</t>
-  </si>
-  <si>
-    <t>Department Name</t>
-  </si>
-  <si>
-    <t>Client Name</t>
-  </si>
-  <si>
-    <t>Payroll Group</t>
-  </si>
-  <si>
-    <t>Cut-Off 1</t>
-  </si>
-  <si>
-    <t>EOM 1</t>
-  </si>
-  <si>
-    <t>Cut-Off 2</t>
-  </si>
-  <si>
-    <t>EOM 2</t>
-  </si>
-  <si>
-    <t>Cut-Off 3</t>
-  </si>
-  <si>
-    <t>EOM 3</t>
-  </si>
-  <si>
-    <t>Cut-Off 4</t>
-  </si>
-  <si>
-    <t>EOM 4</t>
-  </si>
-  <si>
-    <t>Shift Name</t>
-  </si>
-  <si>
-    <t>Shift Type</t>
-  </si>
-  <si>
-    <t>AMIN</t>
-  </si>
-  <si>
-    <t>AM Out</t>
-  </si>
-  <si>
-    <t>PM In</t>
-  </si>
-  <si>
-    <t>PM OUT</t>
-  </si>
-  <si>
-    <t>Break Duration</t>
-  </si>
-  <si>
-    <t>Max Working Minutes</t>
-  </si>
-  <si>
-    <t>PaidLunchBreak</t>
-  </si>
-  <si>
     <t>SalaryType</t>
   </si>
   <si>
+    <t>Hire Date</t>
+  </si>
+  <si>
+    <t>SSS</t>
+  </si>
+  <si>
+    <t>PHIC</t>
+  </si>
+  <si>
+    <t>HDMF</t>
+  </si>
+  <si>
     <t>Daily Rate</t>
   </si>
   <si>
-    <t>Hire Date</t>
-  </si>
-  <si>
-    <t>SSS</t>
-  </si>
-  <si>
-    <t>PHIC</t>
-  </si>
-  <si>
-    <t>HDMF</t>
+    <t>Variable</t>
+  </si>
+  <si>
+    <t>Cut-Off1</t>
+  </si>
+  <si>
+    <t>Cut-Off2</t>
+  </si>
+  <si>
+    <t>Cut-Off3</t>
+  </si>
+  <si>
+    <t>Cut-Off4</t>
+  </si>
+  <si>
+    <t>Semi-Monthly</t>
+  </si>
+  <si>
+    <t>Weekly</t>
+  </si>
+  <si>
+    <t>EOM1</t>
+  </si>
+  <si>
+    <t>EOM2</t>
+  </si>
+  <si>
+    <t>EOM3</t>
+  </si>
+  <si>
+    <t>EOM4</t>
+  </si>
+  <si>
+    <t>Monthly</t>
   </si>
   <si>
     <t>Email</t>
-  </si>
-  <si>
-    <t>Saturday</t>
-  </si>
-  <si>
-    <t>Sunday</t>
-  </si>
-  <si>
-    <t>Semi-Monthly</t>
-  </si>
-  <si>
-    <t>Daysshift - 08:00-17:00</t>
-  </si>
-  <si>
-    <t>Fixed</t>
-  </si>
-  <si>
-    <t>8:00:00AM</t>
-  </si>
-  <si>
-    <t>Variable</t>
-  </si>
-  <si>
-    <t>Weekly</t>
-  </si>
-  <si>
-    <t>Monthly</t>
   </si>
 </sst>
 </file>
@@ -186,14 +320,14 @@
       <sz val="11"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
-      <charset val="134"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
       <color rgb="FFFF0000"/>
       <name val="Aptos Narrow"/>
-      <charset val="134"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
   </fonts>
@@ -219,16 +353,16 @@
   </cellStyleXfs>
   <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="21" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="21" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
@@ -247,6 +381,12 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <person displayName="jhon cee" id="{178AE33B-3851-45CE-B93D-1C219421A458}" userId="fc318abad359ea5a" providerId="Windows Live"/>
+</personList>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -292,7 +432,7 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Aptos Display"/>
+        <a:latin typeface="Aptos Display" panose="02110004020202020204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="游ゴシック Light"/>
@@ -325,9 +465,26 @@
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font script="Armn" typeface="Arial"/>
+        <a:font script="Bugi" typeface="Leelawadee UI"/>
+        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
+        <a:font script="Java" typeface="Javanese Text"/>
+        <a:font script="Lisu" typeface="Segoe UI"/>
+        <a:font script="Mymr" typeface="Myanmar Text"/>
+        <a:font script="Nkoo" typeface="Ebrima"/>
+        <a:font script="Olck" typeface="Nirmala UI"/>
+        <a:font script="Osma" typeface="Ebrima"/>
+        <a:font script="Phag" typeface="Phagspa"/>
+        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
+        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
+        <a:font script="Syre" typeface="Estrangelo Edessa"/>
+        <a:font script="Sora" typeface="Nirmala UI"/>
+        <a:font script="Tale" typeface="Microsoft Tai Le"/>
+        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
+        <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Aptos Narrow"/>
+        <a:latin typeface="Aptos Narrow" panose="02110004020202020204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="游ゴシック"/>
@@ -360,6 +517,23 @@
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font script="Armn" typeface="Arial"/>
+        <a:font script="Bugi" typeface="Leelawadee UI"/>
+        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
+        <a:font script="Java" typeface="Javanese Text"/>
+        <a:font script="Lisu" typeface="Segoe UI"/>
+        <a:font script="Mymr" typeface="Myanmar Text"/>
+        <a:font script="Nkoo" typeface="Ebrima"/>
+        <a:font script="Olck" typeface="Nirmala UI"/>
+        <a:font script="Osma" typeface="Ebrima"/>
+        <a:font script="Phag" typeface="Phagspa"/>
+        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
+        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
+        <a:font script="Syre" typeface="Estrangelo Edessa"/>
+        <a:font script="Sora" typeface="Nirmala UI"/>
+        <a:font script="Tale" typeface="Microsoft Tai Le"/>
+        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
+        <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -522,52 +696,105 @@
     </a:lnDef>
   </a:objectDefaults>
   <a:extraClrSchemeLst/>
+  <a:extLst>
+    <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{2E142A2C-CD16-42D6-873A-C26D2A0506FA}" vid="{1BDDFF52-6CD6-40A5-AB3C-68EB2F1E4D0A}"/>
+    </a:ext>
+  </a:extLst>
 </a:theme>
 </file>
 
+<file path=xl/threadedComments/threadedComment1.xml><?xml version="1.0" encoding="utf-8"?>
+<ThreadedComments xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <threadedComment ref="A2" dT="2026-02-27T23:33:46.22" personId="{178AE33B-3851-45CE-B93D-1C219421A458}" id="{9BFC5F6E-C6A0-42C0-B8AB-F1F3D1249D2B}">
+    <text xml:space="preserve">This is the biometric ID that must be set on the device </text>
+  </threadedComment>
+  <threadedComment ref="H2" dT="2026-02-27T23:40:49.87" personId="{178AE33B-3851-45CE-B93D-1C219421A458}" id="{79FCC02C-F85F-405C-A566-509890A3EBC9}">
+    <text xml:space="preserve">Enter the day name in the column, or leave it blank if not applicable </text>
+  </threadedComment>
+  <threadedComment ref="I2" dT="2026-02-27T23:40:49.87" personId="{178AE33B-3851-45CE-B93D-1C219421A458}" id="{06C68CE5-F9F3-46D3-97DC-8969C057FDE5}">
+    <text xml:space="preserve">Enter the day name in the column, or leave it blank if not applicable </text>
+  </threadedComment>
+  <threadedComment ref="N2" dT="2026-09-14T09:01:47.50" personId="{178AE33B-3851-45CE-B93D-1C219421A458}" id="{96EB2AF4-8857-453C-84CF-C7D0294A47E1}">
+    <text>End of Month</text>
+  </threadedComment>
+  <threadedComment ref="P2" dT="2026-09-14T09:01:47.50" personId="{178AE33B-3851-45CE-B93D-1C219421A458}" id="{ED936B87-B4EA-49D2-9847-251F065AD106}">
+    <text>End of Month</text>
+  </threadedComment>
+  <threadedComment ref="R2" dT="2026-09-14T09:01:47.50" personId="{178AE33B-3851-45CE-B93D-1C219421A458}" id="{861CEFFE-75F3-4A22-A7B0-DE08527FCA28}">
+    <text>End of Month</text>
+  </threadedComment>
+  <threadedComment ref="T2" dT="2026-09-14T09:01:47.50" personId="{178AE33B-3851-45CE-B93D-1C219421A458}" id="{41A77145-9368-44AE-B73E-F2FA9D9BF935}">
+    <text>End of Month</text>
+  </threadedComment>
+  <threadedComment ref="U2" dT="2026-02-27T23:55:36.90" personId="{178AE33B-3851-45CE-B93D-1C219421A458}" id="{73102409-9A79-496E-AAB6-27215C458146}">
+    <text>You can Enter any Time Shift name here</text>
+  </threadedComment>
+  <threadedComment ref="W2" dT="2026-02-27T23:59:32.14" personId="{178AE33B-3851-45CE-B93D-1C219421A458}" id="{C3B48641-F285-4034-95EA-970F81F494AD}">
+    <text xml:space="preserve">Use the same time format shown here. For example, enter 08:00:00 for 8:00 AM and 17:00:00 for 5:00 PM. If the time crosses into the next day, prefix it with 1. before the time. For instance, 1.01:00:00 represents 1:00 AM on the following day. </text>
+  </threadedComment>
+  <threadedComment ref="Y2" dT="2026-02-28T00:02:04.50" personId="{178AE33B-3851-45CE-B93D-1C219421A458}" id="{A1D30F49-4CC7-4810-8930-31A0E5E3D18D}">
+    <text xml:space="preserve">Use the same time format shown here. For example, enter 08:00:00 for 8:00 AM and 17:00:00 for 5:00 PM. If the time crosses into the next day, prefix it with 1. before the time. For instance, 1.01:00:00 represents 1:00 AM on the following day. </text>
+  </threadedComment>
+  <threadedComment ref="Z2" dT="2026-02-28T00:02:10.16" personId="{178AE33B-3851-45CE-B93D-1C219421A458}" id="{0D448524-4E4F-4A1C-9A6D-66C1E154C2FC}">
+    <text xml:space="preserve">Use the same time format shown here. For example, enter 08:00:00 for 8:00 AM and 17:00:00 for 5:00 PM. If the time crosses into the next day, prefix it with 1. before the time. For instance, 1.01:00:00 represents 1:00 AM on the following day. 
+</text>
+  </threadedComment>
+  <threadedComment ref="AB2" dT="2026-02-28T00:09:02.95" personId="{178AE33B-3851-45CE-B93D-1C219421A458}" id="{B19BC939-9062-41D8-A080-1F0317F4D29D}">
+    <text xml:space="preserve">This field represents the total working minutes in a day, excluding unpaid breaks. For example, 480 minutes correspond to 8 hours. If an employee is on a compressed schedule, such as 9 hours per day, you must enter the calculation (9 × 60 = 540) to reflect the correct total. </text>
+  </threadedComment>
+  <threadedComment ref="AD2" dT="2026-02-28T00:29:11.91" personId="{178AE33B-3851-45CE-B93D-1C219421A458}" id="{F0E96506-AAF2-49B7-AD58-D5B640AC0623}">
+    <text xml:space="preserve">The Salary Type column defines how an employee’s salary is calculated for the payroll period. It determines whether the computation is based on actual work hours or on a fixed monthly rate.
+Daily and Monthly Variable: Salary is computed based on the employee’s recorded work hours. This means pay is directly tied to attendance and the number of hours worked within the period.
+Monthly Fixed: Salary is calculated based on the employee’s fixed monthly rate. Deductions are applied for lateness, undertime (UT), and absences, but the base salary remains constant regardless of daily work hours.
+By specifying the correct salary type, the system ensures accurate payroll processing and compliance with company policies
+</text>
+  </threadedComment>
+</ThreadedComments>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{38D9F31A-E2EC-4988-BBA0-8862FC76D1CC}">
   <dimension ref="A1:AJ6"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5" x14ac:dyDescent="0.15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="14" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="11.875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="10.875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="8.875" bestFit="1" customWidth="1"/>
-    <col min="6" max="7" width="6.875" bestFit="1" customWidth="1"/>
-    <col min="8" max="9" width="10.875" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="16" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="11.875" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="14" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="9.875" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="5.875" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="9.875" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="5.875" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="9.875" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="5.875" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="9.875" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="5.875" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="24.25" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="10.875" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="9.875" style="1" customWidth="1"/>
-    <col min="24" max="26" width="8.875" style="1" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="15" style="2" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="20.125" style="3" bestFit="1" customWidth="1"/>
-    <col min="29" max="29" width="15" bestFit="1" customWidth="1"/>
-    <col min="30" max="31" width="10.875" bestFit="1" customWidth="1"/>
-    <col min="32" max="32" width="9.875" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="3.875" bestFit="1" customWidth="1"/>
-    <col min="34" max="35" width="4.875" bestFit="1" customWidth="1"/>
-    <col min="36" max="36" width="5.875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="14.5703125" customWidth="1"/>
+    <col min="2" max="2" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="12.28515625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="9.85546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="5.7109375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="7.28515625" bestFit="1" customWidth="1"/>
+    <col min="8" max="9" width="9.85546875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="17.28515625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="11.7109375" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="13.140625" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="8.140625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="6" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="8.140625" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="6" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="8.140625" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="6" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="8.140625" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="6" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="20.85546875" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="11.7109375" customWidth="1"/>
+    <col min="23" max="23" width="9.85546875" style="2" bestFit="1" customWidth="1"/>
+    <col min="24" max="26" width="8.140625" style="2" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="14.28515625" style="4" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="20" style="3" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="15.42578125" bestFit="1" customWidth="1"/>
+    <col min="30" max="30" width="18.85546875" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="18.85546875" customWidth="1"/>
+    <col min="32" max="32" width="15.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:36" ht="39" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A1" s="4" t="s">
-        <v>0</v>
+    <row r="1" spans="1:36" ht="39" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="6" t="s">
+        <v>2</v>
       </c>
       <c r="B1" s="7" t="s">
-        <v>1</v>
+        <v>27</v>
       </c>
       <c r="C1" s="7"/>
       <c r="D1" s="7"/>
@@ -599,128 +826,128 @@
       <c r="AD1" s="5"/>
       <c r="AE1" s="5"/>
     </row>
-    <row r="2" spans="1:36" x14ac:dyDescent="0.15">
+    <row r="2" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B2" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C2" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D2" t="s">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="E2" t="s">
+        <v>0</v>
+      </c>
+      <c r="F2" t="s">
         <v>6</v>
       </c>
-      <c r="F2" t="s">
+      <c r="G2" t="s">
         <v>7</v>
       </c>
-      <c r="G2" t="s">
+      <c r="H2" t="s">
         <v>8</v>
       </c>
-      <c r="H2" t="s">
+      <c r="I2" t="s">
         <v>9</v>
       </c>
-      <c r="I2" t="s">
+      <c r="J2" t="s">
         <v>10</v>
       </c>
-      <c r="J2" t="s">
+      <c r="K2" t="s">
         <v>11</v>
       </c>
-      <c r="K2" t="s">
+      <c r="L2" t="s">
         <v>12</v>
       </c>
-      <c r="L2" t="s">
+      <c r="M2" t="s">
+        <v>35</v>
+      </c>
+      <c r="N2" t="s">
+        <v>41</v>
+      </c>
+      <c r="O2" t="s">
+        <v>36</v>
+      </c>
+      <c r="P2" t="s">
+        <v>42</v>
+      </c>
+      <c r="Q2" t="s">
+        <v>37</v>
+      </c>
+      <c r="R2" t="s">
+        <v>43</v>
+      </c>
+      <c r="S2" t="s">
+        <v>38</v>
+      </c>
+      <c r="T2" t="s">
+        <v>44</v>
+      </c>
+      <c r="U2" t="s">
         <v>13</v>
       </c>
-      <c r="M2" t="s">
+      <c r="V2" t="s">
         <v>14</v>
       </c>
-      <c r="N2" t="s">
+      <c r="W2" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="O2" t="s">
+      <c r="X2" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="P2" t="s">
+      <c r="Y2" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="Q2" t="s">
+      <c r="Z2" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="R2" t="s">
+      <c r="AA2" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="S2" t="s">
+      <c r="AB2" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="T2" t="s">
+      <c r="AC2" t="s">
         <v>21</v>
       </c>
-      <c r="U2" t="s">
-        <v>22</v>
-      </c>
-      <c r="V2" t="s">
-        <v>23</v>
-      </c>
-      <c r="W2" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="X2" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="Y2" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="Z2" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="AA2" s="2" t="s">
+      <c r="AD2" t="s">
         <v>28</v>
       </c>
-      <c r="AB2" s="3" t="s">
+      <c r="AE2" t="s">
+        <v>33</v>
+      </c>
+      <c r="AF2" t="s">
         <v>29</v>
       </c>
-      <c r="AC2" t="s">
+      <c r="AG2" t="s">
         <v>30</v>
       </c>
-      <c r="AD2" t="s">
+      <c r="AH2" t="s">
         <v>31</v>
       </c>
-      <c r="AE2" t="s">
+      <c r="AI2" t="s">
         <v>32</v>
       </c>
-      <c r="AF2" t="s">
-        <v>33</v>
-      </c>
-      <c r="AG2" t="s">
-        <v>34</v>
-      </c>
-      <c r="AH2" t="s">
-        <v>35</v>
-      </c>
-      <c r="AI2" t="s">
-        <v>36</v>
-      </c>
       <c r="AJ2" t="s">
-        <v>37</v>
+        <v>46</v>
       </c>
     </row>
-    <row r="3" spans="1:36" x14ac:dyDescent="0.15">
+    <row r="3" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>1</v>
       </c>
       <c r="H3" t="s">
-        <v>38</v>
+        <v>22</v>
       </c>
       <c r="I3" t="s">
+        <v>23</v>
+      </c>
+      <c r="L3" t="s">
         <v>39</v>
-      </c>
-      <c r="L3" t="s">
-        <v>40</v>
       </c>
       <c r="M3">
         <v>1</v>
@@ -741,39 +968,39 @@
         <v>0</v>
       </c>
       <c r="U3" t="s">
-        <v>41</v>
+        <v>25</v>
       </c>
       <c r="V3" t="s">
-        <v>42</v>
-      </c>
-      <c r="W3" s="6" t="s">
-        <v>43</v>
-      </c>
-      <c r="X3" s="6">
+        <v>24</v>
+      </c>
+      <c r="W3" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="X3" s="1">
         <v>0.5</v>
       </c>
-      <c r="Y3" s="6">
-        <v>0.54166666666666696</v>
-      </c>
-      <c r="Z3" s="6">
-        <v>0.70833333333333304</v>
-      </c>
-      <c r="AA3" s="2">
+      <c r="Y3" s="1">
+        <v>0.54166666666666663</v>
+      </c>
+      <c r="Z3" s="1">
+        <v>0.70833333333333337</v>
+      </c>
+      <c r="AA3" s="4">
         <v>60</v>
       </c>
-      <c r="AB3" s="2">
+      <c r="AB3" s="4">
         <v>480</v>
       </c>
       <c r="AC3" t="b">
         <v>1</v>
       </c>
       <c r="AD3" t="s">
-        <v>44</v>
+        <v>34</v>
       </c>
     </row>
-    <row r="4" spans="1:36" x14ac:dyDescent="0.15">
+    <row r="4" spans="1:36" x14ac:dyDescent="0.25">
       <c r="L4" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="M4">
         <v>10</v>
@@ -794,9 +1021,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:36" x14ac:dyDescent="0.15">
+    <row r="5" spans="1:36" x14ac:dyDescent="0.25">
       <c r="L5" t="s">
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="M5">
         <v>7</v>
@@ -823,9 +1050,9 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:36" x14ac:dyDescent="0.15">
+    <row r="6" spans="1:36" x14ac:dyDescent="0.25">
       <c r="L6" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="M6">
         <v>31</v>
@@ -839,5 +1066,6 @@
     <mergeCell ref="B1:AC1"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <legacyDrawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add DTR and Payroll Run posting approval flows with deletion-approval cycles
Introduces DTRBatch as a real header entity with its own posting approval
cycle (Save Draft -> Approve/Decline), plus a second approval cycle for
deleting an already-posted DTR or Payroll batch instead of a hard block.
Payroll Run approval is redesigned to match: PayrollBatch gains the same
PendingDeletion/RequestedDeletionByEmployeeId fields and a batch-list
endpoint. GET payrolls also gains an optional payrollBatchId filter so
Payroll Summary can be scoped to one exact run instead of a date range.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/hrms-api/wwwroot/Templates/employee_template.xlsx
+++ b/hrms-api/wwwroot/Templates/employee_template.xlsx
@@ -249,7 +249,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="55">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="57">
   <si>
     <t>Instructions:</t>
   </si>
@@ -388,6 +388,12 @@
   </si>
   <si>
     <t>Address 2</t>
+  </si>
+  <si>
+    <t>Project Site</t>
+  </si>
+  <si>
+    <t>Cash Bond</t>
   </si>
   <si>
     <t>Saturday</t>
@@ -1391,7 +1397,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:AR6"/>
+  <dimension ref="A1:AT6"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.25" outlineLevelRow="5"/>
   <cols>
     <col min="1" max="1" width="14.5666666666667" customWidth="1"/>
@@ -1424,9 +1430,11 @@
     <col min="33" max="33" width="15.2833333333333" customWidth="1"/>
     <col min="39" max="39" width="11.875" customWidth="1"/>
     <col min="40" max="40" width="17.625" customWidth="1"/>
+    <col min="45" max="45" width="11.375" customWidth="1"/>
+    <col min="46" max="46" width="13.875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="39" customHeight="1" spans="1:44">
+    <row r="1" ht="39" customHeight="1" spans="1:46">
       <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
@@ -1464,7 +1472,7 @@
       <c r="AE1" s="5"/>
       <c r="AF1" s="5"/>
     </row>
-    <row r="2" spans="1:44">
+    <row r="2" spans="1:46">
       <c r="A2" t="s">
         <v>2</v>
       </c>
@@ -1597,19 +1605,25 @@
       <c r="AR2" t="s">
         <v>45</v>
       </c>
+      <c r="AS2" t="s">
+        <v>46</v>
+      </c>
+      <c r="AT2" t="s">
+        <v>47</v>
+      </c>
     </row>
-    <row r="3" spans="1:44">
+    <row r="3" spans="1:46">
       <c r="A3">
         <v>1</v>
       </c>
       <c r="H3" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="I3" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="L3" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="M3">
         <v>1</v>
@@ -1630,13 +1644,13 @@
         <v>0</v>
       </c>
       <c r="U3" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="V3" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="W3" s="6" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="X3" s="6">
         <v>0.5</v>
@@ -1657,12 +1671,12 @@
         <v>1</v>
       </c>
       <c r="AD3" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
     </row>
-    <row r="4" spans="1:44">
+    <row r="4" spans="1:46">
       <c r="L4" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="M4">
         <v>10</v>
@@ -1683,9 +1697,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:44">
+    <row r="5" spans="1:46">
       <c r="L5" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="M5">
         <v>7</v>
@@ -1712,9 +1726,9 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:44">
+    <row r="6" spans="1:46">
       <c r="L6" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="M6">
         <v>31</v>

</xml_diff>